<commit_message>
fix: improve q1 workbook compatibility
</commit_message>
<xml_diff>
--- a/results/结果提交模板_Q1_已填写.xlsx
+++ b/results/结果提交模板_Q1_已填写.xlsx
@@ -1086,150 +1086,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Q1BatchDetail" displayName="Q1BatchDetail" ref="A1:V19" headerRowCount="1">
-  <autoFilter ref="A1:V19"/>
-  <tableColumns count="22">
-    <tableColumn id="1" name="架次编号"/>
-    <tableColumn id="2" name="服务区编号"/>
-    <tableColumn id="3" name="机型编号"/>
-    <tableColumn id="4" name="货箱数"/>
-    <tableColumn id="5" name="货箱编号列表"/>
-    <tableColumn id="6" name="总质量_kg"/>
-    <tableColumn id="7" name="安全载荷_kg"/>
-    <tableColumn id="8" name="质量余量_kg"/>
-    <tableColumn id="9" name="质量利用率_%"/>
-    <tableColumn id="10" name="总体积_m3"/>
-    <tableColumn id="11" name="机型体积上限_m3"/>
-    <tableColumn id="12" name="体积余量_m3"/>
-    <tableColumn id="13" name="体积利用率_%"/>
-    <tableColumn id="14" name="单程距离_m"/>
-    <tableColumn id="15" name="往返距离_m"/>
-    <tableColumn id="16" name="安全载荷对应航程_m"/>
-    <tableColumn id="17" name="航程余量_m"/>
-    <tableColumn id="18" name="架次能耗_kWh"/>
-    <tableColumn id="19" name="允许任务能量_kWh"/>
-    <tableColumn id="20" name="能耗占允许_%"/>
-    <tableColumn id="21" name="往返时间_s"/>
-    <tableColumn id="22" name="返航SOC_%"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Q1MethodCompare" displayName="Q1MethodCompare" ref="A1:M5" headerRowCount="1">
-  <autoFilter ref="A1:M5"/>
-  <tableColumns count="13">
-    <tableColumn id="1" name="方法"/>
-    <tableColumn id="2" name="架次数"/>
-    <tableColumn id="3" name="架次节省_架"/>
-    <tableColumn id="4" name="架次节省_%"/>
-    <tableColumn id="5" name="总运输能耗_kWh"/>
-    <tableColumn id="6" name="能耗节省_kWh"/>
-    <tableColumn id="7" name="能耗节省_%"/>
-    <tableColumn id="8" name="累计作业时间_s"/>
-    <tableColumn id="9" name="时间节省_s"/>
-    <tableColumn id="10" name="时间节省_%"/>
-    <tableColumn id="11" name="搜索是否完整"/>
-    <tableColumn id="12" name="约束验证"/>
-    <tableColumn id="13" name="说明"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Q1SafePayload" displayName="Q1SafePayload" ref="A1:N46" headerRowCount="1">
-  <autoFilter ref="A1:N46"/>
-  <tableColumns count="14">
-    <tableColumn id="1" name="机型编号"/>
-    <tableColumn id="2" name="服务区编号"/>
-    <tableColumn id="3" name="返航余量ρ"/>
-    <tableColumn id="4" name="最大安全载荷_kg"/>
-    <tableColumn id="5" name="额定最大载荷_kg"/>
-    <tableColumn id="6" name="安全载荷占额定_%"/>
-    <tableColumn id="7" name="往返能耗_kWh"/>
-    <tableColumn id="8" name="允许任务能量_kWh"/>
-    <tableColumn id="9" name="能量余量_kWh"/>
-    <tableColumn id="10" name="往返距离_m"/>
-    <tableColumn id="11" name="安全载荷对应航程_m"/>
-    <tableColumn id="12" name="航程余量_m"/>
-    <tableColumn id="13" name="零载荷是否可行"/>
-    <tableColumn id="14" name="搜索方法"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Q1Sensitivity" displayName="Q1Sensitivity" ref="A1:P6" headerRowCount="1">
-  <autoFilter ref="A1:P6"/>
-  <tableColumns count="16">
-    <tableColumn id="1" name="返航余量ρ"/>
-    <tableColumn id="2" name="FFD架次"/>
-    <tableColumn id="3" name="局部搜索架次"/>
-    <tableColumn id="4" name="架次节省_架"/>
-    <tableColumn id="5" name="FFD能耗_kWh"/>
-    <tableColumn id="6" name="局部搜索能耗_kWh"/>
-    <tableColumn id="7" name="局部搜索相对FFD节能_%"/>
-    <tableColumn id="8" name="FFD时间_s"/>
-    <tableColumn id="9" name="局部搜索时间_s"/>
-    <tableColumn id="10" name="A型最小安全载荷_kg"/>
-    <tableColumn id="11" name="B型最小安全载荷_kg"/>
-    <tableColumn id="12" name="C型最小安全载荷_kg"/>
-    <tableColumn id="13" name="A型受限服务区数"/>
-    <tableColumn id="14" name="B型受限服务区数"/>
-    <tableColumn id="15" name="C型受限服务区数"/>
-    <tableColumn id="16" name="相对上一ρ变化"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Q1Validation" displayName="Q1Validation" ref="A1:N5" headerRowCount="1">
-  <autoFilter ref="A1:N5"/>
-  <tableColumns count="14">
-    <tableColumn id="1" name="方法"/>
-    <tableColumn id="2" name="架次数"/>
-    <tableColumn id="3" name="货箱数"/>
-    <tableColumn id="4" name="搜索是否完整"/>
-    <tableColumn id="5" name="总体通过"/>
-    <tableColumn id="6" name="箱体唯一覆盖"/>
-    <tableColumn id="7" name="不跨服务区"/>
-    <tableColumn id="8" name="质量容量"/>
-    <tableColumn id="9" name="体积容量"/>
-    <tableColumn id="10" name="能耗余量"/>
-    <tableColumn id="11" name="航程约束"/>
-    <tableColumn id="12" name="总量一致"/>
-    <tableColumn id="13" name="有限数值"/>
-    <tableColumn id="14" name="备注"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Q1RouteGeometry" displayName="Q1RouteGeometry" ref="A1:K16" headerRowCount="1">
-  <autoFilter ref="A1:K16"/>
-  <tableColumns count="11">
-    <tableColumn id="1" name="服务区编号"/>
-    <tableColumn id="2" name="单程距离_m"/>
-    <tableColumn id="3" name="最高地面高程_m"/>
-    <tableColumn id="4" name="巡航海拔_m"/>
-    <tableColumn id="5" name="去程爬升_m"/>
-    <tableColumn id="6" name="去程下降_m"/>
-    <tableColumn id="7" name="返程爬升_m"/>
-    <tableColumn id="8" name="返程下降_m"/>
-    <tableColumn id="9" name="A_往返飞行时间_s"/>
-    <tableColumn id="10" name="B_往返飞行时间_s"/>
-    <tableColumn id="11" name="C_往返飞行时间_s"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
   <a:themeElements>
@@ -3986,9 +3842,6 @@
   </sheetData>
   <autoFilter ref="A1:N46"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -4364,9 +4217,6 @@
   </sheetData>
   <autoFilter ref="A1:P6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -4742,9 +4592,6 @@
   </sheetData>
   <autoFilter ref="A1:N5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -5685,9 +5532,6 @@
   </sheetData>
   <autoFilter ref="A1:K16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -11743,9 +11587,6 @@
   </sheetData>
   <autoFilter ref="A1:V19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -12039,8 +11880,5 @@
   </sheetData>
   <autoFilter ref="A1:M5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>